<commit_message>
Load and RES generation plot functions added.
</commit_message>
<xml_diff>
--- a/data/CS7/case33_1/case33_1_operational_data.xlsx
+++ b/data/CS7/case33_1/case33_1_operational_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\thesis-shared-resources-planning-no_esso-degradation\data\CS7\case33_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15FFD224-F604-415F-B2EE-D7A0614E0C54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98E4449F-1B44-4BB5-B025-7F7EB23EE700}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20295" yWindow="-20640" windowWidth="28800" windowHeight="15285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-15195" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Characterization" sheetId="2" r:id="rId1"/>
@@ -1036,7 +1036,7 @@
         <v>8</v>
       </c>
       <c r="C30" s="1">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="D30" s="2">
         <v>5.3835800807536999E-2</v>

</xml_diff>